<commit_message>
implemented authetification and reworked db schema
</commit_message>
<xml_diff>
--- a/Doku/zeitplan_HungerSatt.xlsx
+++ b/Doku/zeitplan_HungerSatt.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://htlsaalfelden322-my.sharepoint.com/personal/johannes_ellmer_htl-saalfelden_at/Documents/Dokumente/GitHub/Diplomarbeit_Bestellapp/Doku/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="100" documentId="8_{3460CF72-AC89-4CED-8824-3C5C9549F2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F08F4E60-AAE5-49AB-B84A-C81A912A30C3}"/>
+  <xr:revisionPtr revIDLastSave="105" documentId="8_{3460CF72-AC89-4CED-8824-3C5C9549F2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1611B18-63A8-416F-8866-5CF8DB4104C6}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{72F4632B-4B3C-4A8B-9C92-C659B892C97E}"/>
   </bookViews>
@@ -168,7 +168,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,6 +199,13 @@
     <font>
       <sz val="11"/>
       <color theme="5" tint="0.39997558519241921"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -237,7 +244,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
+        <fgColor rgb="FF0070C0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -589,7 +596,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -644,7 +651,60 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -660,12 +720,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -684,54 +738,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1178,65 +1186,65 @@
       <c r="AD19" s="9"/>
     </row>
     <row r="20" spans="1:34" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A20" s="61" t="s">
+      <c r="A20" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="61"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="66" t="s">
+      <c r="B20" s="45"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="E20" s="67"/>
-      <c r="F20" s="66" t="s">
+      <c r="E20" s="51"/>
+      <c r="F20" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="59"/>
-      <c r="H20" s="59"/>
-      <c r="I20" s="59" t="s">
+      <c r="G20" s="43"/>
+      <c r="H20" s="43"/>
+      <c r="I20" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="J20" s="59"/>
-      <c r="K20" s="59"/>
-      <c r="L20" s="59"/>
-      <c r="M20" s="59"/>
-      <c r="N20" s="59" t="s">
+      <c r="J20" s="43"/>
+      <c r="K20" s="43"/>
+      <c r="L20" s="43"/>
+      <c r="M20" s="43"/>
+      <c r="N20" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="O20" s="59"/>
-      <c r="P20" s="59"/>
-      <c r="Q20" s="59"/>
-      <c r="R20" s="59" t="s">
+      <c r="O20" s="43"/>
+      <c r="P20" s="43"/>
+      <c r="Q20" s="43"/>
+      <c r="R20" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="S20" s="59"/>
-      <c r="T20" s="59"/>
-      <c r="U20" s="59"/>
-      <c r="V20" s="59" t="s">
+      <c r="S20" s="43"/>
+      <c r="T20" s="43"/>
+      <c r="U20" s="43"/>
+      <c r="V20" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="W20" s="59"/>
-      <c r="X20" s="59"/>
-      <c r="Y20" s="59"/>
-      <c r="Z20" s="59" t="s">
+      <c r="W20" s="43"/>
+      <c r="X20" s="43"/>
+      <c r="Y20" s="43"/>
+      <c r="Z20" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="AA20" s="59"/>
-      <c r="AB20" s="59"/>
-      <c r="AC20" s="59"/>
-      <c r="AD20" s="60"/>
-      <c r="AE20" s="55" t="s">
+      <c r="AA20" s="43"/>
+      <c r="AB20" s="43"/>
+      <c r="AC20" s="43"/>
+      <c r="AD20" s="44"/>
+      <c r="AE20" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="AF20" s="55"/>
-      <c r="AG20" s="55"/>
-      <c r="AH20" s="56"/>
+      <c r="AF20" s="38"/>
+      <c r="AG20" s="38"/>
+      <c r="AH20" s="39"/>
     </row>
     <row r="21" spans="1:34" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A21" s="63" t="s">
+      <c r="A21" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="64"/>
-      <c r="C21" s="65"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="49"/>
       <c r="D21" s="22" t="s">
         <v>3</v>
       </c>
@@ -1332,11 +1340,11 @@
       </c>
     </row>
     <row r="22" spans="1:34" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="44" t="s">
+      <c r="A22" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="40"/>
       <c r="D22" s="7">
         <v>2</v>
       </c>
@@ -1348,11 +1356,11 @@
       <c r="AH22" s="8"/>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A23" s="44" t="s">
+      <c r="A23" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="44"/>
-      <c r="C23" s="44"/>
+      <c r="B23" s="40"/>
+      <c r="C23" s="40"/>
       <c r="D23" s="7">
         <v>10</v>
       </c>
@@ -1365,11 +1373,11 @@
       <c r="AH23" s="8"/>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A24" s="44" t="s">
+      <c r="A24" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="44"/>
-      <c r="C24" s="44"/>
+      <c r="B24" s="40"/>
+      <c r="C24" s="40"/>
       <c r="D24" s="7">
         <v>5</v>
       </c>
@@ -1380,11 +1388,11 @@
       <c r="AH24" s="8"/>
     </row>
     <row r="25" spans="1:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A25" s="57" t="s">
+      <c r="A25" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="57"/>
-      <c r="C25" s="58"/>
+      <c r="B25" s="41"/>
+      <c r="C25" s="42"/>
       <c r="D25" s="15">
         <f>SUM(D22:D24)</f>
         <v>17</v>
@@ -1438,8 +1446,8 @@
       <c r="I26" s="37"/>
       <c r="L26" s="37"/>
       <c r="M26" s="37"/>
-      <c r="N26" s="38"/>
-      <c r="O26" s="38"/>
+      <c r="N26" s="67"/>
+      <c r="O26" s="67"/>
       <c r="AH26" s="8"/>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.45">
@@ -1460,11 +1468,11 @@
       <c r="AH27" s="8"/>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A28" s="44" t="s">
+      <c r="A28" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="44"/>
-      <c r="C28" s="45"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="54"/>
       <c r="D28">
         <v>9</v>
       </c>
@@ -1480,11 +1488,11 @@
       <c r="AH28" s="8"/>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A29" s="44" t="s">
+      <c r="A29" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="44"/>
-      <c r="C29" s="44"/>
+      <c r="B29" s="40"/>
+      <c r="C29" s="40"/>
       <c r="D29" s="7">
         <v>8</v>
       </c>
@@ -1495,11 +1503,11 @@
       <c r="AH29" s="8"/>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A30" s="44" t="s">
+      <c r="A30" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="44"/>
-      <c r="C30" s="45"/>
+      <c r="B30" s="40"/>
+      <c r="C30" s="54"/>
       <c r="D30">
         <v>10</v>
       </c>
@@ -1511,11 +1519,11 @@
       <c r="AH30" s="8"/>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A31" s="44" t="s">
+      <c r="A31" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="B31" s="44"/>
-      <c r="C31" s="44"/>
+      <c r="B31" s="40"/>
+      <c r="C31" s="40"/>
       <c r="D31" s="7">
         <v>10</v>
       </c>
@@ -1528,11 +1536,11 @@
       <c r="AH31" s="8"/>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A32" s="44" t="s">
+      <c r="A32" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="44"/>
-      <c r="C32" s="44"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="40"/>
       <c r="D32" s="7">
         <v>0</v>
       </c>
@@ -1546,11 +1554,11 @@
       <c r="AH32" s="8"/>
     </row>
     <row r="33" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A33" s="54" t="s">
+      <c r="A33" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="54"/>
-      <c r="C33" s="54"/>
+      <c r="B33" s="55"/>
+      <c r="C33" s="55"/>
       <c r="D33" s="17">
         <v>4</v>
       </c>
@@ -1605,11 +1613,11 @@
       <c r="AH34" s="8"/>
     </row>
     <row r="35" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A35" s="44" t="s">
+      <c r="A35" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="B35" s="44"/>
-      <c r="C35" s="44"/>
+      <c r="B35" s="40"/>
+      <c r="C35" s="40"/>
       <c r="D35" s="7">
         <v>0</v>
       </c>
@@ -1621,11 +1629,11 @@
       <c r="AH35" s="8"/>
     </row>
     <row r="36" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A36" s="44" t="s">
+      <c r="A36" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="44"/>
-      <c r="C36" s="45"/>
+      <c r="B36" s="40"/>
+      <c r="C36" s="54"/>
       <c r="D36">
         <v>0</v>
       </c>
@@ -1637,11 +1645,11 @@
       <c r="AH36" s="8"/>
     </row>
     <row r="37" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A37" s="44" t="s">
+      <c r="A37" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B37" s="44"/>
-      <c r="C37" s="45"/>
+      <c r="B37" s="40"/>
+      <c r="C37" s="54"/>
       <c r="D37">
         <v>15</v>
       </c>
@@ -1654,11 +1662,11 @@
       <c r="AH37" s="8"/>
     </row>
     <row r="38" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A38" s="44" t="s">
+      <c r="A38" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="B38" s="44"/>
-      <c r="C38" s="45"/>
+      <c r="B38" s="40"/>
+      <c r="C38" s="54"/>
       <c r="D38">
         <v>10</v>
       </c>
@@ -1671,11 +1679,11 @@
       <c r="AH38" s="8"/>
     </row>
     <row r="39" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A39" s="44" t="s">
+      <c r="A39" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="44"/>
-      <c r="C39" s="45"/>
+      <c r="B39" s="40"/>
+      <c r="C39" s="54"/>
       <c r="D39">
         <v>5</v>
       </c>
@@ -1689,11 +1697,11 @@
       <c r="AH39" s="10"/>
     </row>
     <row r="40" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="46" t="s">
+      <c r="A40" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="B40" s="47"/>
-      <c r="C40" s="48"/>
+      <c r="B40" s="62"/>
+      <c r="C40" s="63"/>
       <c r="D40" s="18">
         <f>SUM(D41:D43)</f>
         <v>38</v>
@@ -1777,11 +1785,11 @@
       <c r="AI43" s="7"/>
     </row>
     <row r="44" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A44" s="49" t="s">
+      <c r="A44" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="B44" s="50"/>
-      <c r="C44" s="51"/>
+      <c r="B44" s="65"/>
+      <c r="C44" s="66"/>
       <c r="D44" s="18">
         <f>SUM(D45:D46)</f>
         <v>15</v>
@@ -1876,11 +1884,11 @@
       <c r="AH46" s="10"/>
     </row>
     <row r="47" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="39" t="s">
+      <c r="A47" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="B47" s="39"/>
-      <c r="C47" s="40"/>
+      <c r="B47" s="56"/>
+      <c r="C47" s="57"/>
       <c r="D47" s="4">
         <v>60</v>
       </c>
@@ -1891,11 +1899,11 @@
       <c r="AH47" s="8"/>
     </row>
     <row r="48" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A48" s="44" t="s">
+      <c r="A48" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="44"/>
-      <c r="C48" s="45"/>
+      <c r="B48" s="40"/>
+      <c r="C48" s="54"/>
       <c r="D48">
         <v>18</v>
       </c>
@@ -1922,8 +1930,9 @@
       </c>
       <c r="L49" s="29"/>
       <c r="M49" s="29"/>
-      <c r="N49" s="5"/>
+      <c r="N49" s="68"/>
       <c r="O49" s="5"/>
+      <c r="U49" s="5"/>
       <c r="V49" s="5"/>
       <c r="AB49" s="5"/>
       <c r="AC49" s="5"/>
@@ -1931,11 +1940,11 @@
       <c r="AH49" s="8"/>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A50" s="41" t="s">
+      <c r="A50" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="B50" s="42"/>
-      <c r="C50" s="43"/>
+      <c r="B50" s="59"/>
+      <c r="C50" s="60"/>
       <c r="D50" s="35">
         <f>D25+D26+D27+D34+D40+D44+D47</f>
         <v>211</v>
@@ -1980,6 +1989,24 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
     <mergeCell ref="AE20:AH20"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A23:C23"/>
@@ -1994,24 +2021,6 @@
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="I20:M20"/>
     <mergeCell ref="N20:Q20"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A37:C37"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactor: clean up comments and improve order status formatting in user profile
</commit_message>
<xml_diff>
--- a/Doku/zeitplan_HungerSatt.xlsx
+++ b/Doku/zeitplan_HungerSatt.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://htlsaalfelden322-my.sharepoint.com/personal/johannes_ellmer_htl-saalfelden_at/Documents/Dokumente/GitHub/Diplomarbeit_Bestellapp/Doku/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="8_{3460CF72-AC89-4CED-8824-3C5C9549F2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1611B18-63A8-416F-8866-5CF8DB4104C6}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="8_{3460CF72-AC89-4CED-8824-3C5C9549F2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B09B3C56-FD6D-4F14-9EC3-E174EC62E951}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{72F4632B-4B3C-4A8B-9C92-C659B892C97E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>HungerSatt Online-Bestellservice</t>
   </si>
@@ -162,6 +162,15 @@
   </si>
   <si>
     <t>Hosting Planen</t>
+  </si>
+  <si>
+    <t>Geändertes Ziel / fällt weg</t>
+  </si>
+  <si>
+    <t>Offen</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -211,7 +220,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -244,7 +253,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0070C0"/>
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -596,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -651,15 +666,60 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -693,53 +753,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1186,65 +1202,65 @@
       <c r="AD19" s="9"/>
     </row>
     <row r="20" spans="1:34" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A20" s="45" t="s">
+      <c r="A20" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="45"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="50" t="s">
+      <c r="B20" s="60"/>
+      <c r="C20" s="61"/>
+      <c r="D20" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="E20" s="51"/>
-      <c r="F20" s="50" t="s">
+      <c r="E20" s="66"/>
+      <c r="F20" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="43"/>
-      <c r="H20" s="43"/>
-      <c r="I20" s="43" t="s">
+      <c r="G20" s="58"/>
+      <c r="H20" s="58"/>
+      <c r="I20" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="J20" s="43"/>
-      <c r="K20" s="43"/>
-      <c r="L20" s="43"/>
-      <c r="M20" s="43"/>
-      <c r="N20" s="43" t="s">
+      <c r="J20" s="58"/>
+      <c r="K20" s="58"/>
+      <c r="L20" s="58"/>
+      <c r="M20" s="58"/>
+      <c r="N20" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="O20" s="43"/>
-      <c r="P20" s="43"/>
-      <c r="Q20" s="43"/>
-      <c r="R20" s="43" t="s">
+      <c r="O20" s="58"/>
+      <c r="P20" s="58"/>
+      <c r="Q20" s="58"/>
+      <c r="R20" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="S20" s="43"/>
-      <c r="T20" s="43"/>
-      <c r="U20" s="43"/>
-      <c r="V20" s="43" t="s">
+      <c r="S20" s="58"/>
+      <c r="T20" s="58"/>
+      <c r="U20" s="58"/>
+      <c r="V20" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="W20" s="43"/>
-      <c r="X20" s="43"/>
-      <c r="Y20" s="43"/>
-      <c r="Z20" s="43" t="s">
+      <c r="W20" s="58"/>
+      <c r="X20" s="58"/>
+      <c r="Y20" s="58"/>
+      <c r="Z20" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="AA20" s="43"/>
-      <c r="AB20" s="43"/>
-      <c r="AC20" s="43"/>
-      <c r="AD20" s="44"/>
-      <c r="AE20" s="38" t="s">
+      <c r="AA20" s="58"/>
+      <c r="AB20" s="58"/>
+      <c r="AC20" s="58"/>
+      <c r="AD20" s="59"/>
+      <c r="AE20" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="AF20" s="38"/>
-      <c r="AG20" s="38"/>
-      <c r="AH20" s="39"/>
+      <c r="AF20" s="54"/>
+      <c r="AG20" s="54"/>
+      <c r="AH20" s="55"/>
     </row>
     <row r="21" spans="1:34" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A21" s="47" t="s">
+      <c r="A21" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="48"/>
-      <c r="C21" s="49"/>
+      <c r="B21" s="63"/>
+      <c r="C21" s="64"/>
       <c r="D21" s="22" t="s">
         <v>3</v>
       </c>
@@ -1340,11 +1356,11 @@
       </c>
     </row>
     <row r="22" spans="1:34" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
       <c r="D22" s="7">
         <v>2</v>
       </c>
@@ -1356,11 +1372,11 @@
       <c r="AH22" s="8"/>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A23" s="40" t="s">
+      <c r="A23" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="40"/>
-      <c r="C23" s="40"/>
+      <c r="B23" s="43"/>
+      <c r="C23" s="43"/>
       <c r="D23" s="7">
         <v>10</v>
       </c>
@@ -1373,11 +1389,11 @@
       <c r="AH23" s="8"/>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A24" s="40" t="s">
+      <c r="A24" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="40"/>
-      <c r="C24" s="40"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="43"/>
       <c r="D24" s="7">
         <v>5</v>
       </c>
@@ -1388,11 +1404,11 @@
       <c r="AH24" s="8"/>
     </row>
     <row r="25" spans="1:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A25" s="41" t="s">
+      <c r="A25" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="41"/>
-      <c r="C25" s="42"/>
+      <c r="B25" s="56"/>
+      <c r="C25" s="57"/>
       <c r="D25" s="15">
         <f>SUM(D22:D24)</f>
         <v>17</v>
@@ -1446,16 +1462,16 @@
       <c r="I26" s="37"/>
       <c r="L26" s="37"/>
       <c r="M26" s="37"/>
-      <c r="N26" s="67"/>
-      <c r="O26" s="67"/>
+      <c r="N26" s="68"/>
+      <c r="O26" s="68"/>
       <c r="AH26" s="8"/>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A27" s="52" t="s">
+      <c r="A27" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="52"/>
-      <c r="C27" s="53"/>
+      <c r="B27" s="51"/>
+      <c r="C27" s="52"/>
       <c r="D27" s="4">
         <f>SUM(D28:D33)</f>
         <v>41</v>
@@ -1468,11 +1484,11 @@
       <c r="AH27" s="8"/>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A28" s="40" t="s">
+      <c r="A28" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="40"/>
-      <c r="C28" s="54"/>
+      <c r="B28" s="43"/>
+      <c r="C28" s="44"/>
       <c r="D28">
         <v>9</v>
       </c>
@@ -1488,11 +1504,11 @@
       <c r="AH28" s="8"/>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A29" s="40" t="s">
+      <c r="A29" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="40"/>
-      <c r="C29" s="40"/>
+      <c r="B29" s="43"/>
+      <c r="C29" s="43"/>
       <c r="D29" s="7">
         <v>8</v>
       </c>
@@ -1503,11 +1519,11 @@
       <c r="AH29" s="8"/>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A30" s="40" t="s">
+      <c r="A30" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="40"/>
-      <c r="C30" s="54"/>
+      <c r="B30" s="43"/>
+      <c r="C30" s="44"/>
       <c r="D30">
         <v>10</v>
       </c>
@@ -1516,14 +1532,18 @@
       </c>
       <c r="J30" s="29"/>
       <c r="K30" s="29"/>
+      <c r="Z30" s="69"/>
+      <c r="AA30" t="s">
+        <v>42</v>
+      </c>
       <c r="AH30" s="8"/>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A31" s="40" t="s">
+      <c r="A31" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="B31" s="40"/>
-      <c r="C31" s="40"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="43"/>
       <c r="D31" s="7">
         <v>10</v>
       </c>
@@ -1536,11 +1556,11 @@
       <c r="AH31" s="8"/>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A32" s="40" t="s">
+      <c r="A32" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
       <c r="D32" s="7">
         <v>0</v>
       </c>
@@ -1551,14 +1571,18 @@
       <c r="K32" s="29"/>
       <c r="L32" s="29"/>
       <c r="M32" s="29"/>
+      <c r="Z32" s="5"/>
+      <c r="AA32" t="s">
+        <v>43</v>
+      </c>
       <c r="AH32" s="8"/>
     </row>
     <row r="33" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A33" s="55" t="s">
+      <c r="A33" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="55"/>
-      <c r="C33" s="55"/>
+      <c r="B33" s="53"/>
+      <c r="C33" s="53"/>
       <c r="D33" s="17">
         <v>4</v>
       </c>
@@ -1571,7 +1595,7 @@
       <c r="I33" s="9"/>
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
-      <c r="L33" s="15"/>
+      <c r="L33" s="30"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9"/>
       <c r="O33" s="9"/>
@@ -1596,11 +1620,11 @@
       <c r="AH33" s="10"/>
     </row>
     <row r="34" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="52" t="s">
+      <c r="A34" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="52"/>
-      <c r="C34" s="53"/>
+      <c r="B34" s="51"/>
+      <c r="C34" s="52"/>
       <c r="D34" s="4">
         <f>SUM(D35:D39)</f>
         <v>30</v>
@@ -1611,13 +1635,16 @@
       </c>
       <c r="M34" s="6"/>
       <c r="AH34" s="8"/>
+      <c r="AI34" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="35" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A35" s="40" t="s">
+      <c r="A35" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="B35" s="40"/>
-      <c r="C35" s="40"/>
+      <c r="B35" s="43"/>
+      <c r="C35" s="43"/>
       <c r="D35" s="7">
         <v>0</v>
       </c>
@@ -1625,15 +1652,15 @@
         <v>10</v>
       </c>
       <c r="N35" s="29"/>
-      <c r="O35" s="5"/>
+      <c r="O35" s="29"/>
       <c r="AH35" s="8"/>
     </row>
     <row r="36" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A36" s="40" t="s">
+      <c r="A36" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="40"/>
-      <c r="C36" s="54"/>
+      <c r="B36" s="43"/>
+      <c r="C36" s="44"/>
       <c r="D36">
         <v>0</v>
       </c>
@@ -1641,15 +1668,15 @@
         <v>15</v>
       </c>
       <c r="O36" s="29"/>
-      <c r="P36" s="5"/>
+      <c r="P36" s="29"/>
       <c r="AH36" s="8"/>
     </row>
     <row r="37" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A37" s="40" t="s">
+      <c r="A37" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="B37" s="40"/>
-      <c r="C37" s="54"/>
+      <c r="B37" s="43"/>
+      <c r="C37" s="44"/>
       <c r="D37">
         <v>15</v>
       </c>
@@ -1658,15 +1685,15 @@
       </c>
       <c r="N37" s="29"/>
       <c r="O37" s="29"/>
-      <c r="P37" s="5"/>
+      <c r="P37" s="29"/>
       <c r="AH37" s="8"/>
     </row>
     <row r="38" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A38" s="40" t="s">
+      <c r="A38" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="B38" s="40"/>
-      <c r="C38" s="54"/>
+      <c r="B38" s="43"/>
+      <c r="C38" s="44"/>
       <c r="D38">
         <v>10</v>
       </c>
@@ -1679,29 +1706,29 @@
       <c r="AH38" s="8"/>
     </row>
     <row r="39" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A39" s="40" t="s">
+      <c r="A39" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="40"/>
-      <c r="C39" s="54"/>
+      <c r="B39" s="43"/>
+      <c r="C39" s="44"/>
       <c r="D39">
         <v>5</v>
       </c>
       <c r="E39" s="8">
         <v>1</v>
       </c>
-      <c r="O39" s="5"/>
+      <c r="O39" s="29"/>
       <c r="AE39" s="9"/>
       <c r="AF39" s="9"/>
       <c r="AG39" s="9"/>
       <c r="AH39" s="10"/>
     </row>
     <row r="40" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="61" t="s">
+      <c r="A40" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="B40" s="62"/>
-      <c r="C40" s="63"/>
+      <c r="B40" s="46"/>
+      <c r="C40" s="47"/>
       <c r="D40" s="18">
         <f>SUM(D41:D43)</f>
         <v>38</v>
@@ -1748,7 +1775,7 @@
       <c r="E41" s="8">
         <v>6</v>
       </c>
-      <c r="R41" s="5"/>
+      <c r="R41" s="67"/>
       <c r="AH41" s="8"/>
     </row>
     <row r="42" spans="1:35" x14ac:dyDescent="0.45">
@@ -1762,7 +1789,7 @@
       <c r="E42" s="8">
         <v>10</v>
       </c>
-      <c r="S42" s="5"/>
+      <c r="S42" s="67"/>
       <c r="AH42" s="8"/>
     </row>
     <row r="43" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -1776,8 +1803,8 @@
       <c r="E43" s="8">
         <v>10</v>
       </c>
-      <c r="S43" s="5"/>
-      <c r="T43" s="5"/>
+      <c r="S43" s="67"/>
+      <c r="T43" s="67"/>
       <c r="AE43" s="9"/>
       <c r="AF43" s="9"/>
       <c r="AG43" s="9"/>
@@ -1785,11 +1812,11 @@
       <c r="AI43" s="7"/>
     </row>
     <row r="44" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A44" s="64" t="s">
+      <c r="A44" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="B44" s="65"/>
-      <c r="C44" s="66"/>
+      <c r="B44" s="49"/>
+      <c r="C44" s="50"/>
       <c r="D44" s="18">
         <f>SUM(D45:D46)</f>
         <v>15</v>
@@ -1837,8 +1864,9 @@
         <v>4</v>
       </c>
       <c r="F45" s="7"/>
-      <c r="W45" s="5"/>
-      <c r="X45" s="5"/>
+      <c r="W45" s="29"/>
+      <c r="X45" s="29"/>
+      <c r="Y45" s="29"/>
       <c r="AH45" s="8"/>
     </row>
     <row r="46" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -1872,8 +1900,8 @@
       <c r="V46" s="9"/>
       <c r="W46" s="9"/>
       <c r="X46" s="9"/>
-      <c r="Y46" s="15"/>
-      <c r="Z46" s="15"/>
+      <c r="Y46" s="30"/>
+      <c r="Z46" s="30"/>
       <c r="AA46" s="9"/>
       <c r="AB46" s="9"/>
       <c r="AC46" s="9"/>
@@ -1884,33 +1912,33 @@
       <c r="AH46" s="10"/>
     </row>
     <row r="47" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="56" t="s">
+      <c r="A47" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="B47" s="56"/>
-      <c r="C47" s="57"/>
+      <c r="B47" s="38"/>
+      <c r="C47" s="39"/>
       <c r="D47" s="4">
         <v>60</v>
       </c>
       <c r="E47" s="14">
         <v>65</v>
       </c>
-      <c r="Z47" s="5"/>
+      <c r="Z47" s="69"/>
       <c r="AH47" s="8"/>
     </row>
     <row r="48" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A48" s="40" t="s">
+      <c r="A48" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="40"/>
-      <c r="C48" s="54"/>
+      <c r="B48" s="43"/>
+      <c r="C48" s="44"/>
       <c r="D48">
         <v>18</v>
       </c>
       <c r="E48" s="8">
         <v>23</v>
       </c>
-      <c r="Y48" s="5"/>
+      <c r="Y48" s="29"/>
       <c r="Z48" s="5"/>
       <c r="AA48" s="5"/>
       <c r="AB48" s="5"/>
@@ -1930,21 +1958,21 @@
       </c>
       <c r="L49" s="29"/>
       <c r="M49" s="29"/>
-      <c r="N49" s="68"/>
-      <c r="O49" s="5"/>
-      <c r="U49" s="5"/>
-      <c r="V49" s="5"/>
+      <c r="N49" s="29"/>
+      <c r="O49" s="29"/>
+      <c r="U49" s="29"/>
+      <c r="V49" s="29"/>
       <c r="AB49" s="5"/>
       <c r="AC49" s="5"/>
       <c r="AD49" s="5"/>
       <c r="AH49" s="8"/>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A50" s="58" t="s">
+      <c r="A50" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="B50" s="59"/>
-      <c r="C50" s="60"/>
+      <c r="B50" s="41"/>
+      <c r="C50" s="42"/>
       <c r="D50" s="35">
         <f>D25+D26+D27+D34+D40+D44+D47</f>
         <v>211</v>
@@ -1989,24 +2017,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
     <mergeCell ref="AE20:AH20"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A23:C23"/>
@@ -2021,6 +2031,24 @@
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="I20:M20"/>
     <mergeCell ref="N20:Q20"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A37:C37"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update order time and add new documentation files
</commit_message>
<xml_diff>
--- a/Doku/zeitplan_HungerSatt.xlsx
+++ b/Doku/zeitplan_HungerSatt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://htlsaalfelden322-my.sharepoint.com/personal/johannes_ellmer_htl-saalfelden_at/Documents/Dokumente/GitHub/Diplomarbeit_Bestellapp/Doku/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="142" documentId="8_{3460CF72-AC89-4CED-8824-3C5C9549F2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E784B1CF-927A-4A45-B05D-2A1A36C26875}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="8_{3460CF72-AC89-4CED-8824-3C5C9549F2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0100F7D-0C2B-4334-93A9-90354C55CB88}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{72F4632B-4B3C-4A8B-9C92-C659B892C97E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{72F4632B-4B3C-4A8B-9C92-C659B892C97E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>HungerSatt Online-Bestellservice</t>
   </si>
@@ -168,9 +168,6 @@
   </si>
   <si>
     <t>Offen</t>
-  </si>
-  <si>
-    <t>x</t>
   </si>
 </sst>
 </file>
@@ -227,7 +224,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -260,12 +257,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -618,7 +609,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -673,18 +664,63 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -718,52 +754,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1165,22 +1155,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{875DED61-2A9A-40C9-A51B-4495B2B330E0}">
   <dimension ref="A1:AI51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.265625" customWidth="1"/>
     <col min="6" max="34" width="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" s="2"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A3" s="1"/>
     </row>
-    <row r="19" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
@@ -1209,66 +1199,66 @@
       <c r="AC19" s="9"/>
       <c r="AD19" s="9"/>
     </row>
-    <row r="20" spans="1:34" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="48" t="s">
+    <row r="20" spans="1:34" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A20" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="48"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="53" t="s">
+      <c r="B20" s="63"/>
+      <c r="C20" s="64"/>
+      <c r="D20" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="E20" s="54"/>
-      <c r="F20" s="53" t="s">
+      <c r="E20" s="69"/>
+      <c r="F20" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46" t="s">
+      <c r="G20" s="61"/>
+      <c r="H20" s="61"/>
+      <c r="I20" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="J20" s="46"/>
-      <c r="K20" s="46"/>
-      <c r="L20" s="46"/>
-      <c r="M20" s="46"/>
-      <c r="N20" s="46" t="s">
+      <c r="J20" s="61"/>
+      <c r="K20" s="61"/>
+      <c r="L20" s="61"/>
+      <c r="M20" s="61"/>
+      <c r="N20" s="61" t="s">
         <v>7</v>
       </c>
-      <c r="O20" s="46"/>
-      <c r="P20" s="46"/>
-      <c r="Q20" s="46"/>
-      <c r="R20" s="46" t="s">
+      <c r="O20" s="61"/>
+      <c r="P20" s="61"/>
+      <c r="Q20" s="61"/>
+      <c r="R20" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="S20" s="46"/>
-      <c r="T20" s="46"/>
-      <c r="U20" s="46"/>
-      <c r="V20" s="46" t="s">
+      <c r="S20" s="61"/>
+      <c r="T20" s="61"/>
+      <c r="U20" s="61"/>
+      <c r="V20" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="W20" s="46"/>
-      <c r="X20" s="46"/>
-      <c r="Y20" s="46"/>
-      <c r="Z20" s="46" t="s">
+      <c r="W20" s="61"/>
+      <c r="X20" s="61"/>
+      <c r="Y20" s="61"/>
+      <c r="Z20" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="AA20" s="46"/>
-      <c r="AB20" s="46"/>
-      <c r="AC20" s="46"/>
-      <c r="AD20" s="47"/>
-      <c r="AE20" s="41" t="s">
+      <c r="AA20" s="61"/>
+      <c r="AB20" s="61"/>
+      <c r="AC20" s="61"/>
+      <c r="AD20" s="62"/>
+      <c r="AE20" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="AF20" s="41"/>
-      <c r="AG20" s="41"/>
-      <c r="AH20" s="42"/>
-    </row>
-    <row r="21" spans="1:34" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="50" t="s">
+      <c r="AF20" s="57"/>
+      <c r="AG20" s="57"/>
+      <c r="AH20" s="58"/>
+    </row>
+    <row r="21" spans="1:34" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A21" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="51"/>
-      <c r="C21" s="52"/>
+      <c r="B21" s="66"/>
+      <c r="C21" s="67"/>
       <c r="D21" s="22" t="s">
         <v>3</v>
       </c>
@@ -1363,12 +1353,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:34" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+    <row r="22" spans="1:34" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="43"/>
-      <c r="C22" s="43"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
       <c r="D22" s="7">
         <v>2</v>
       </c>
@@ -1379,12 +1369,12 @@
       <c r="G22" s="29"/>
       <c r="AH22" s="8"/>
     </row>
-    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A23" s="43" t="s">
+    <row r="23" spans="1:34" x14ac:dyDescent="0.45">
+      <c r="A23" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="43"/>
+      <c r="B23" s="46"/>
+      <c r="C23" s="46"/>
       <c r="D23" s="7">
         <v>10</v>
       </c>
@@ -1396,12 +1386,12 @@
       <c r="H23" s="29"/>
       <c r="AH23" s="8"/>
     </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A24" s="43" t="s">
+    <row r="24" spans="1:34" x14ac:dyDescent="0.45">
+      <c r="A24" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
       <c r="D24" s="7">
         <v>5</v>
       </c>
@@ -1411,12 +1401,12 @@
       <c r="H24" s="29"/>
       <c r="AH24" s="8"/>
     </row>
-    <row r="25" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="44" t="s">
+    <row r="25" spans="1:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A25" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="44"/>
-      <c r="C25" s="45"/>
+      <c r="B25" s="59"/>
+      <c r="C25" s="60"/>
       <c r="D25" s="15">
         <f>SUM(D22:D24)</f>
         <v>17</v>
@@ -1455,7 +1445,7 @@
       <c r="AG25" s="9"/>
       <c r="AH25" s="10"/>
     </row>
-    <row r="26" spans="1:34" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:34" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
         <v>16</v>
       </c>
@@ -1470,16 +1460,16 @@
       <c r="I26" s="37"/>
       <c r="L26" s="37"/>
       <c r="M26" s="37"/>
-      <c r="N26" s="39"/>
-      <c r="O26" s="39"/>
+      <c r="N26" s="38"/>
+      <c r="O26" s="38"/>
       <c r="AH26" s="8"/>
     </row>
-    <row r="27" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A27" s="55" t="s">
+    <row r="27" spans="1:34" x14ac:dyDescent="0.45">
+      <c r="A27" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="55"/>
-      <c r="C27" s="56"/>
+      <c r="B27" s="54"/>
+      <c r="C27" s="55"/>
       <c r="D27" s="4">
         <f>SUM(D28:D33)</f>
         <v>41</v>
@@ -1491,12 +1481,12 @@
       <c r="I27" s="29"/>
       <c r="AH27" s="8"/>
     </row>
-    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A28" s="43" t="s">
+    <row r="28" spans="1:34" x14ac:dyDescent="0.45">
+      <c r="A28" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="43"/>
-      <c r="C28" s="57"/>
+      <c r="B28" s="46"/>
+      <c r="C28" s="47"/>
       <c r="D28">
         <v>9</v>
       </c>
@@ -1511,12 +1501,12 @@
       </c>
       <c r="AH28" s="8"/>
     </row>
-    <row r="29" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A29" s="43" t="s">
+    <row r="29" spans="1:34" x14ac:dyDescent="0.45">
+      <c r="A29" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="43"/>
-      <c r="C29" s="43"/>
+      <c r="B29" s="46"/>
+      <c r="C29" s="46"/>
       <c r="D29" s="7">
         <v>8</v>
       </c>
@@ -1526,12 +1516,12 @@
       <c r="I29" s="29"/>
       <c r="AH29" s="8"/>
     </row>
-    <row r="30" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A30" s="43" t="s">
+    <row r="30" spans="1:34" x14ac:dyDescent="0.45">
+      <c r="A30" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="43"/>
-      <c r="C30" s="57"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="47"/>
       <c r="D30">
         <v>10</v>
       </c>
@@ -1540,18 +1530,18 @@
       </c>
       <c r="J30" s="29"/>
       <c r="K30" s="29"/>
-      <c r="Z30" s="40"/>
+      <c r="Z30" s="39"/>
       <c r="AA30" t="s">
         <v>42</v>
       </c>
       <c r="AH30" s="8"/>
     </row>
-    <row r="31" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A31" s="43" t="s">
+    <row r="31" spans="1:34" x14ac:dyDescent="0.45">
+      <c r="A31" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="B31" s="43"/>
-      <c r="C31" s="43"/>
+      <c r="B31" s="46"/>
+      <c r="C31" s="46"/>
       <c r="D31" s="7">
         <v>10</v>
       </c>
@@ -1563,12 +1553,12 @@
       <c r="K31" s="29"/>
       <c r="AH31" s="8"/>
     </row>
-    <row r="32" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A32" s="43" t="s">
+    <row r="32" spans="1:34" x14ac:dyDescent="0.45">
+      <c r="A32" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="43"/>
+      <c r="B32" s="46"/>
+      <c r="C32" s="46"/>
       <c r="D32" s="7">
         <v>0</v>
       </c>
@@ -1585,12 +1575,12 @@
       </c>
       <c r="AH32" s="8"/>
     </row>
-    <row r="33" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="58" t="s">
+    <row r="33" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A33" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="58"/>
-      <c r="C33" s="58"/>
+      <c r="B33" s="56"/>
+      <c r="C33" s="56"/>
       <c r="D33" s="17">
         <v>4</v>
       </c>
@@ -1627,12 +1617,12 @@
       <c r="AG33" s="9"/>
       <c r="AH33" s="10"/>
     </row>
-    <row r="34" spans="1:35" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="55" t="s">
+    <row r="34" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="55"/>
-      <c r="C34" s="56"/>
+      <c r="B34" s="54"/>
+      <c r="C34" s="55"/>
       <c r="D34" s="4">
         <f>SUM(D35:D39)</f>
         <v>30</v>
@@ -1643,16 +1633,13 @@
       </c>
       <c r="M34" s="6"/>
       <c r="AH34" s="8"/>
-      <c r="AI34" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A35" s="43" t="s">
+    </row>
+    <row r="35" spans="1:35" x14ac:dyDescent="0.45">
+      <c r="A35" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="B35" s="43"/>
-      <c r="C35" s="43"/>
+      <c r="B35" s="46"/>
+      <c r="C35" s="46"/>
       <c r="D35" s="7">
         <v>0</v>
       </c>
@@ -1663,12 +1650,12 @@
       <c r="O35" s="29"/>
       <c r="AH35" s="8"/>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A36" s="43" t="s">
+    <row r="36" spans="1:35" x14ac:dyDescent="0.45">
+      <c r="A36" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="43"/>
-      <c r="C36" s="57"/>
+      <c r="B36" s="46"/>
+      <c r="C36" s="47"/>
       <c r="D36">
         <v>0</v>
       </c>
@@ -1677,14 +1664,15 @@
       </c>
       <c r="O36" s="29"/>
       <c r="P36" s="29"/>
+      <c r="Q36" s="29"/>
       <c r="AH36" s="8"/>
     </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A37" s="43" t="s">
+    <row r="37" spans="1:35" x14ac:dyDescent="0.45">
+      <c r="A37" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="B37" s="43"/>
-      <c r="C37" s="57"/>
+      <c r="B37" s="46"/>
+      <c r="C37" s="47"/>
       <c r="D37">
         <v>15</v>
       </c>
@@ -1696,12 +1684,12 @@
       <c r="P37" s="29"/>
       <c r="AH37" s="8"/>
     </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A38" s="43" t="s">
+    <row r="38" spans="1:35" x14ac:dyDescent="0.45">
+      <c r="A38" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="B38" s="43"/>
-      <c r="C38" s="57"/>
+      <c r="B38" s="46"/>
+      <c r="C38" s="47"/>
       <c r="D38">
         <v>10</v>
       </c>
@@ -1711,15 +1699,15 @@
       <c r="O38" s="29"/>
       <c r="P38" s="29"/>
       <c r="Q38" s="29"/>
-      <c r="R38" s="70"/>
+      <c r="R38" s="40"/>
       <c r="AH38" s="8"/>
     </row>
-    <row r="39" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="43" t="s">
+    <row r="39" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A39" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="43"/>
-      <c r="C39" s="57"/>
+      <c r="B39" s="46"/>
+      <c r="C39" s="47"/>
       <c r="D39">
         <v>5</v>
       </c>
@@ -1732,12 +1720,12 @@
       <c r="AG39" s="9"/>
       <c r="AH39" s="10"/>
     </row>
-    <row r="40" spans="1:35" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="64" t="s">
+    <row r="40" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A40" s="48" t="s">
         <v>29</v>
       </c>
-      <c r="B40" s="65"/>
-      <c r="C40" s="66"/>
+      <c r="B40" s="49"/>
+      <c r="C40" s="50"/>
       <c r="D40" s="18">
         <f>SUM(D41:D43)</f>
         <v>38</v>
@@ -1773,7 +1761,7 @@
       <c r="AD40" s="13"/>
       <c r="AH40" s="8"/>
     </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>28</v>
       </c>
@@ -1784,10 +1772,10 @@
       <c r="E41" s="8">
         <v>6</v>
       </c>
-      <c r="R41" s="38"/>
+      <c r="R41" s="39"/>
       <c r="AH41" s="8"/>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>37</v>
       </c>
@@ -1798,10 +1786,10 @@
       <c r="E42" s="8">
         <v>10</v>
       </c>
-      <c r="S42" s="38"/>
+      <c r="S42" s="39"/>
       <c r="AH42" s="8"/>
     </row>
-    <row r="43" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A43" t="s">
         <v>30</v>
       </c>
@@ -1812,20 +1800,20 @@
       <c r="E43" s="8">
         <v>10</v>
       </c>
-      <c r="S43" s="38"/>
-      <c r="T43" s="38"/>
+      <c r="S43" s="39"/>
+      <c r="T43" s="39"/>
       <c r="AE43" s="9"/>
       <c r="AF43" s="9"/>
       <c r="AG43" s="9"/>
       <c r="AH43" s="9"/>
       <c r="AI43" s="7"/>
     </row>
-    <row r="44" spans="1:35" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="67" t="s">
+    <row r="44" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A44" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="B44" s="68"/>
-      <c r="C44" s="69"/>
+      <c r="B44" s="52"/>
+      <c r="C44" s="53"/>
       <c r="D44" s="18">
         <f>SUM(D45:D46)</f>
         <v>15</v>
@@ -1861,7 +1849,7 @@
       <c r="AD44" s="13"/>
       <c r="AH44" s="8"/>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>40</v>
       </c>
@@ -1873,12 +1861,13 @@
         <v>4</v>
       </c>
       <c r="F45" s="7"/>
+      <c r="V45" s="39"/>
       <c r="W45" s="29"/>
       <c r="X45" s="29"/>
       <c r="Y45" s="29"/>
       <c r="AH45" s="8"/>
     </row>
-    <row r="46" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:35" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A46" s="9" t="s">
         <v>32</v>
       </c>
@@ -1908,7 +1897,7 @@
       <c r="U46" s="9"/>
       <c r="V46" s="9"/>
       <c r="W46" s="9"/>
-      <c r="X46" s="9"/>
+      <c r="X46" s="39"/>
       <c r="Y46" s="30"/>
       <c r="Z46" s="30"/>
       <c r="AA46" s="9"/>
@@ -1920,44 +1909,45 @@
       <c r="AG46" s="9"/>
       <c r="AH46" s="10"/>
     </row>
-    <row r="47" spans="1:35" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="59" t="s">
+    <row r="47" spans="1:35" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A47" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="60"/>
+      <c r="B47" s="41"/>
+      <c r="C47" s="42"/>
       <c r="D47" s="4">
         <v>60</v>
       </c>
       <c r="E47" s="14">
         <v>65</v>
       </c>
-      <c r="Z47" s="40"/>
+      <c r="Y47" s="39"/>
+      <c r="Z47" s="39"/>
       <c r="AH47" s="8"/>
     </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A48" s="43" t="s">
+    <row r="48" spans="1:35" x14ac:dyDescent="0.45">
+      <c r="A48" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="43"/>
-      <c r="C48" s="57"/>
+      <c r="B48" s="46"/>
+      <c r="C48" s="47"/>
       <c r="D48">
         <v>18</v>
       </c>
       <c r="E48" s="8">
         <v>23</v>
       </c>
-      <c r="Y48" s="5"/>
-      <c r="Z48" s="5"/>
-      <c r="AA48" s="5"/>
+      <c r="Y48" s="29"/>
+      <c r="Z48" s="29"/>
+      <c r="AA48" s="29"/>
       <c r="AB48" s="29"/>
-      <c r="AC48" s="5"/>
+      <c r="AC48" s="29"/>
       <c r="AE48" s="29"/>
       <c r="AF48" s="29"/>
       <c r="AG48" s="29"/>
       <c r="AH48" s="8"/>
     </row>
-    <row r="49" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A49" t="s">
         <v>34</v>
       </c>
@@ -1976,18 +1966,18 @@
       <c r="V49" s="29"/>
       <c r="AB49" s="29"/>
       <c r="AC49" s="29"/>
-      <c r="AD49" s="5"/>
+      <c r="AD49" s="29"/>
       <c r="AE49" s="29"/>
       <c r="AF49" s="29"/>
-      <c r="AG49" s="5"/>
+      <c r="AG49" s="29"/>
       <c r="AH49" s="8"/>
     </row>
-    <row r="50" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A50" s="61" t="s">
+    <row r="50" spans="1:34" x14ac:dyDescent="0.45">
+      <c r="A50" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="B50" s="62"/>
-      <c r="C50" s="63"/>
+      <c r="B50" s="44"/>
+      <c r="C50" s="45"/>
       <c r="D50" s="35">
         <f>D25+D26+D27+D34+D40+D44+D47</f>
         <v>211</v>
@@ -2026,30 +2016,12 @@
       <c r="AG50" s="31"/>
       <c r="AH50" s="32"/>
     </row>
-    <row r="51" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:34" x14ac:dyDescent="0.45">
       <c r="D51" s="7"/>
       <c r="E51" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
     <mergeCell ref="AE20:AH20"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A23:C23"/>
@@ -2064,6 +2036,24 @@
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="I20:M20"/>
     <mergeCell ref="N20:Q20"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A37:C37"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>